<commit_message>
Working implementation of reading files by chunks Implemented a line counter to restart upload after a given line number (TODO) Found bug in data cleaner where values could be permuted between lines (only appears if lines were sorted)
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24069987-A5EF-4A8A-A797-A1356985606D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3492ED-3BAA-434E-A7CC-B3AA94CFA755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="243">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -856,6 +856,15 @@
   </si>
   <si>
     <t>multi csv files</t>
+  </si>
+  <si>
+    <t>Custom Key Example</t>
+  </si>
+  <si>
+    <t>Test value</t>
+  </si>
+  <si>
+    <t>Custom key-value pair example</t>
   </si>
 </sst>
 </file>
@@ -2148,7 +2157,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C74C64-19A1-4B6C-85B0-52803ED84917}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" style="3" customWidth="1"/>
@@ -2278,6 +2287,17 @@
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel file: added support for parameters __Limit__ __Time between requests__ to adjust data flow to CKAN server (also used via CLI) Implemented print_help_cli functions to display arguments to user Debug builder_resource_datastore_multi_folder
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3492ED-3BAA-434E-A7CC-B3AA94CFA755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5AD468-99E4-4BC7-B604-4164FE70617E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-22440" yWindow="3315" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="245">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -865,6 +865,12 @@
   </si>
   <si>
     <t>Custom key-value pair example</t>
+  </si>
+  <si>
+    <t>Time between requests</t>
+  </si>
+  <si>
+    <t>Time between each request in seconds</t>
   </si>
 </sst>
 </file>
@@ -1334,7 +1340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC716B16-D7ED-4B3B-A67B-512577BD3E75}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1415,6 +1421,17 @@
       </c>
       <c r="C9" t="s">
         <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10">
+        <v>0.1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel file: renamed package __Name__ column to __Name in URL__
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5AD468-99E4-4BC7-B604-4164FE70617E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0A4099-3FCD-4BCF-BAC2-8B2944821548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22440" yWindow="3315" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-23295" yWindow="3750" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="248">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -871,6 +871,15 @@
   </si>
   <si>
     <t>Time between each request in seconds</t>
+  </si>
+  <si>
+    <t>Limit</t>
+  </si>
+  <si>
+    <t>Maximum number of records to return/send per request</t>
+  </si>
+  <si>
+    <t>Name in URL</t>
   </si>
 </sst>
 </file>
@@ -1340,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC716B16-D7ED-4B3B-A67B-512577BD3E75}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1425,12 +1434,23 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B10">
+        <v>1000</v>
+      </c>
+      <c r="C10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>0.1</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>244</v>
       </c>
     </row>
@@ -2196,7 +2216,7 @@
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Excel file: added __Data cleaner__ field for DataStore resources
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0A4099-3FCD-4BCF-BAC2-8B2944821548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC3CC65-1BD9-4FFB-A526-545A8557EE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23295" yWindow="3750" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="253">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -880,6 +880,21 @@
   </si>
   <si>
     <t>Name in URL</t>
+  </si>
+  <si>
+    <t>Data cleaner</t>
+  </si>
+  <si>
+    <t>Data cleaners</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>GeoJSON</t>
   </si>
 </sst>
 </file>
@@ -2369,7 +2384,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016621B7-2234-4AB7-B879-700B37012293}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="39.85546875" customWidth="1"/>
@@ -2382,9 +2397,10 @@
     <col min="9" max="9" width="14.7109375" customWidth="1"/>
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -2419,10 +2435,16 @@
         <v>98</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2450,11 +2472,11 @@
       <c r="K2" t="s">
         <v>100</v>
       </c>
-      <c r="L2" t="s">
+      <c r="N2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -2479,11 +2501,11 @@
       <c r="I3" t="s">
         <v>15</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>86</v>
       </c>
@@ -2500,7 +2522,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>76</v>
       </c>
@@ -2517,7 +2539,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>164</v>
       </c>
@@ -2531,7 +2553,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>118</v>
       </c>
@@ -2548,7 +2570,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>165</v>
       </c>
@@ -2568,7 +2590,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>167</v>
       </c>
@@ -2585,7 +2607,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>195</v>
       </c>
@@ -2612,12 +2634,18 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7E3C6D2E-2102-4413-8B48-F48B66AA0F6D}">
           <x14:formula1>
             <xm:f>validation!$A$43:$A$55</xm:f>
           </x14:formula1>
           <xm:sqref>D1:D1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{49765E69-A9C5-42AE-9CD1-A6196AF2CE5C}">
+          <x14:formula1>
+            <xm:f>validation!$A$58:$A$63</xm:f>
+          </x14:formula1>
+          <xm:sqref>L1:L1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2993,7 +3021,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397C6D0D-9607-4B06-96F5-66D1EA23B080}">
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -3243,51 +3271,73 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="B57" s="14"/>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>6</v>
-      </c>
-      <c r="B58" t="s">
-        <v>228</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>251</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B64" s="14"/>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>72</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A64:B64"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A57:B57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Documentation of the CLI arguments used in various locations Recommendations for dataset metadata (under construction)
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC3CC65-1BD9-4FFB-A526-545A8557EE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D4CEDB-543D-44EA-A6CD-60EC76417673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -849,9 +849,6 @@
 - MultiDataStore: A MultiFile which initiates a DataStore and manages field metadata. The forbidden wildcard characters in the name of the Excel spreadsheet for field metadata must be replaced by `#`.</t>
   </si>
   <si>
-    <t>Name identifying the dataset, used in the URL (short name, lowercase)</t>
-  </si>
-  <si>
     <t>DataStore Columns Sheet</t>
   </si>
   <si>
@@ -895,6 +892,9 @@
   </si>
   <si>
     <t>GeoJSON</t>
+  </si>
+  <si>
+    <t>Name used in the URL to reference the dataset (short name, only accepting lowercase letters (a-z), digits (0-9), `-` and `_`, no accents, no spaces, length 2-100 characters)</t>
   </si>
 </sst>
 </file>
@@ -1449,24 +1449,24 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B10">
         <v>1000</v>
       </c>
       <c r="C10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B11">
         <v>0.1</v>
       </c>
       <c r="C11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -2229,15 +2229,15 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2343,13 +2343,13 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>241</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -2405,7 +2405,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -2435,7 +2435,7 @@
         <v>98</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>208</v>
@@ -2612,7 +2612,7 @@
         <v>195</v>
       </c>
       <c r="B10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
@@ -3271,23 +3271,23 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B57" s="14"/>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Data cleaner: adding a Check mode which does not alter data but raises an exception when a field does not conform to expected formatting TODO: validate
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D4CEDB-543D-44EA-A6CD-60EC76417673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54842A2E-EC84-41F9-A88B-508051F66182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="257">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -895,6 +895,18 @@
   </si>
   <si>
     <t>Name used in the URL to reference the dataset (short name, only accepting lowercase letters (a-z), digits (0-9), `-` and `_`, no accents, no spaces, length 2-100 characters)</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Raises an error before upload if a data is badly formatted</t>
+  </si>
+  <si>
+    <t>Automatically replaces most common data format errors</t>
+  </si>
+  <si>
+    <t>Manages geometric fields conversion and EPSG conversions</t>
   </si>
 </sst>
 </file>
@@ -3284,10 +3296,24 @@
       <c r="A59" t="s">
         <v>250</v>
       </c>
+      <c r="B59" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>251</v>
+      </c>
+      <c r="B60" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>253</v>
+      </c>
+      <c r="B61" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Clearer distinction between metadata from user, data source/data cleaner or pre-existing CKAN metadata Implemented progress callback for the various levels of the tasks
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54842A2E-EC84-41F9-A88B-508051F66182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03193867-FA4F-43CB-9CAD-CC65FE92B0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="28680" yWindow="1755" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -24,6 +24,10 @@
     <sheet name="validation" sheetId="6" r:id="rId9"/>
     <sheet name="help" sheetId="8" r:id="rId10"/>
   </sheets>
+  <definedNames>
+    <definedName name="CKAN_URL">ckan!$B$2</definedName>
+    <definedName name="package_name">package!$B$2</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -913,7 +917,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -942,6 +946,14 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -976,10 +988,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1018,6 +1031,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1043,7 +1059,8 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1499,25 +1516,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" spans="1:3" ht="102" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
     </row>
     <row r="3" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
@@ -1542,10 +1559,10 @@
       <c r="A7" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="C7" s="18"/>
+      <c r="C7" s="19"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
@@ -1606,10 +1623,10 @@
       <c r="A13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="C13" s="19"/>
+      <c r="C13" s="20"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
@@ -1780,10 +1797,10 @@
       <c r="A29" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="C29" s="18"/>
+      <c r="C29" s="19"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
@@ -1877,10 +1894,10 @@
       <c r="A38" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="19" t="s">
+      <c r="B38" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="C38" s="19"/>
+      <c r="C38" s="20"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
@@ -2018,28 +2035,28 @@
       <c r="A51" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="20" t="s">
+      <c r="B51" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="C51" s="20"/>
+      <c r="C51" s="21"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B52" s="21" t="s">
+      <c r="B52" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="C52" s="21"/>
+      <c r="C52" s="22"/>
     </row>
     <row r="53" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B53" s="18" t="s">
+      <c r="B53" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="C53" s="18"/>
+      <c r="C53" s="19"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
@@ -2221,7 +2238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C74C64-19A1-4B6C-85B0-52803ED84917}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" style="3" customWidth="1"/>
@@ -2230,7 +2247,7 @@
     <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>68</v>
       </c>
@@ -2241,7 +2258,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>246</v>
       </c>
@@ -2251,8 +2268,12 @@
       <c r="C2" s="1" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="14" t="str">
+        <f>HYPERLINK(IF(RIGHT(CKAN_URL,1)="/", CKAN_URL &amp; "dataset/" &amp; package_name, CKAN_URL &amp; "/dataset/" &amp; package_name))</f>
+        <v>/dataset/builder-example-py</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -2263,7 +2284,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -2274,7 +2295,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -2282,7 +2303,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
@@ -2293,7 +2314,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
@@ -2301,7 +2322,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -2309,7 +2330,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>23</v>
       </c>
@@ -2317,7 +2338,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>32</v>
       </c>
@@ -2325,7 +2346,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>51</v>
       </c>
@@ -2333,27 +2354,27 @@
         <v>156</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>239</v>
       </c>
@@ -3049,10 +3070,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="14"/>
+      <c r="B2" s="15"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -3065,10 +3086,10 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="15"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -3086,10 +3107,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="14"/>
+      <c r="B13" s="15"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -3152,10 +3173,10 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="14"/>
+      <c r="B34" s="15"/>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
@@ -3188,10 +3209,10 @@
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
+      <c r="A42" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B42" s="14"/>
+      <c r="B42" s="15"/>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
@@ -3282,10 +3303,10 @@
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="14" t="s">
+      <c r="A57" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="B57" s="14"/>
+      <c r="B57" s="15"/>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -3317,10 +3338,10 @@
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="14" t="s">
+      <c r="A64" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B64" s="14"/>
+      <c r="B64" s="15"/>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">

</xml_diff>

<commit_message>
Documentation Added a new default location for the CKAN API key: ~/.config/__CKAN_API_KEY__.txt
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03193867-FA4F-43CB-9CAD-CC65FE92B0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DF5C45-7E3C-4094-B8CA-4ED0D988DF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="257">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -764,9 +764,6 @@
     <t>Names for read only aliases of the resource (only for DataStores).</t>
   </si>
   <si>
-    <t>default</t>
-  </si>
-  <si>
     <t>Index</t>
   </si>
   <si>
@@ -792,18 +789,6 @@
   </si>
   <si>
     <t>bson</t>
-  </si>
-  <si>
-    <t>geometry</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>point</t>
-  </si>
-  <si>
-    <t>polygon</t>
   </si>
   <si>
     <t>float8</t>
@@ -911,6 +896,21 @@
   </si>
   <si>
     <t>Manages geometric fields conversion and EPSG conversions</t>
+  </si>
+  <si>
+    <t>geometry(GEOMETRY,4326)</t>
+  </si>
+  <si>
+    <t>Field accepting GeoJSON (WKB hexadecimal preferred), in WGS84 coordinate system</t>
+  </si>
+  <si>
+    <t>Binary JSON</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Recommended to specify author/maintainer to communicate on the dataset</t>
   </si>
 </sst>
 </file>
@@ -1473,29 +1473,29 @@
         <v>208</v>
       </c>
       <c r="C9" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B10">
         <v>1000</v>
       </c>
       <c r="C10" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B11">
         <v>0.1</v>
       </c>
       <c r="C11" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -1887,7 +1887,7 @@
         <v>208</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -1929,7 +1929,7 @@
         <v>2</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1951,7 +1951,7 @@
         <v>30</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -2107,10 +2107,10 @@
         <v>111</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -2118,10 +2118,10 @@
         <v>111</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -2129,10 +2129,10 @@
         <v>111</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2243,7 +2243,7 @@
   <cols>
     <col min="1" max="1" width="26.85546875" style="3" customWidth="1"/>
     <col min="2" max="2" width="127" style="1" customWidth="1"/>
-    <col min="3" max="3" width="59.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="70.140625" style="1" customWidth="1"/>
     <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
@@ -2258,15 +2258,15 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="D2" s="14" t="str">
         <f>HYPERLINK(IF(RIGHT(CKAN_URL,1)="/", CKAN_URL &amp; "dataset/" &amp; package_name, CKAN_URL &amp; "/dataset/" &amp; package_name))</f>
@@ -2358,6 +2358,9 @@
       <c r="A12" s="3" t="s">
         <v>26</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
@@ -2368,6 +2371,9 @@
       <c r="A14" s="3" t="s">
         <v>28</v>
       </c>
+      <c r="C14" s="1" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
@@ -2376,13 +2382,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2417,28 +2423,27 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016621B7-2234-4AB7-B879-700B37012293}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="39.85546875" customWidth="1"/>
     <col min="3" max="3" width="9.42578125" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.42578125" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" customWidth="1"/>
-    <col min="7" max="7" width="79" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="79" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -2450,34 +2455,31 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>247</v>
-      </c>
       <c r="M1" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="N1" s="2" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2493,23 +2495,20 @@
       <c r="E2" t="s">
         <v>123</v>
       </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
       <c r="G2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" t="s">
         <v>15</v>
       </c>
+      <c r="I2" t="s">
+        <v>99</v>
+      </c>
       <c r="J2" t="s">
-        <v>99</v>
-      </c>
-      <c r="K2" t="s">
         <v>100</v>
       </c>
-      <c r="N2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -2523,22 +2522,19 @@
         <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>233</v>
+        <v>228</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
       </c>
       <c r="G3" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="H3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I3" t="s">
         <v>15</v>
       </c>
-      <c r="N3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>86</v>
       </c>
@@ -2551,11 +2547,11 @@
       <c r="E4" t="s">
         <v>86</v>
       </c>
-      <c r="G4" t="s">
+      <c r="F4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>76</v>
       </c>
@@ -2568,11 +2564,11 @@
       <c r="E5" t="s">
         <v>87</v>
       </c>
-      <c r="G5" t="s">
+      <c r="F5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>164</v>
       </c>
@@ -2582,11 +2578,11 @@
       <c r="D6" t="s">
         <v>137</v>
       </c>
-      <c r="G6" t="s">
+      <c r="F6" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>118</v>
       </c>
@@ -2599,11 +2595,11 @@
       <c r="E7" t="s">
         <v>117</v>
       </c>
-      <c r="G7" t="s">
+      <c r="F7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>165</v>
       </c>
@@ -2616,14 +2612,14 @@
       <c r="D8" t="s">
         <v>138</v>
       </c>
+      <c r="F8" t="s">
+        <v>120</v>
+      </c>
       <c r="G8" t="s">
-        <v>120</v>
-      </c>
-      <c r="H8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>167</v>
       </c>
@@ -2636,16 +2632,16 @@
       <c r="E9" t="s">
         <v>168</v>
       </c>
-      <c r="G9" t="s">
+      <c r="F9" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>195</v>
       </c>
       <c r="B10" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
@@ -2654,31 +2650,34 @@
         <v>197</v>
       </c>
       <c r="E10" t="s">
-        <v>232</v>
-      </c>
-      <c r="G10" t="s">
+        <v>227</v>
+      </c>
+      <c r="F10" t="s">
         <v>198</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" sqref="C1:C1048576" xr:uid="{ABB3E20A-99D1-46AC-9089-895EB5CEC278}"/>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{ABB3E20A-99D1-46AC-9089-895EB5CEC278}">
+          <x14:formula1>
+            <xm:f>validation!$A$62:$A$72</xm:f>
+          </x14:formula1>
+          <xm:sqref>C1:C1048576</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7E3C6D2E-2102-4413-8B48-F48B66AA0F6D}">
           <x14:formula1>
-            <xm:f>validation!$A$43:$A$55</xm:f>
+            <xm:f>validation!$A$40:$A$52</xm:f>
           </x14:formula1>
           <xm:sqref>D1:D1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{49765E69-A9C5-42AE-9CD1-A6196AF2CE5C}">
           <x14:formula1>
-            <xm:f>validation!$A$58:$A$63</xm:f>
+            <xm:f>validation!$A$55:$A$60</xm:f>
           </x14:formula1>
-          <xm:sqref>L1:L1048576</xm:sqref>
+          <xm:sqref>K1:K1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2736,6 +2735,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{AC34424F-01A6-4AC6-A6D2-12548F5B7C2E}">
+          <x14:formula1>
+            <xm:f>validation!$A$14:$A$30</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -2866,6 +2877,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{BACB5A16-C96C-41B9-84A8-2A34CF62D54E}">
+          <x14:formula1>
+            <xm:f>validation!$A$14:$A$30</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -2919,6 +2942,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{A359947D-B60D-4238-867D-215340AE3426}">
+          <x14:formula1>
+            <xm:f>validation!$A$14:$A$30</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -3049,12 +3084,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{7E1D0734-FE78-4DA9-A387-5BA151C3DC93}">
+          <x14:formula1>
+            <xm:f>validation!$A$14:$A$30</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397C6D0D-9607-4B06-96F5-66D1EA23B080}">
-  <dimension ref="A1:B70"/>
+  <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -3127,264 +3174,262 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>227</v>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="15"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B34" s="15"/>
+      <c r="A34" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>141</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>109</v>
+        <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>54</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>55</v>
-      </c>
+      <c r="A39" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="15"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>31</v>
+      </c>
+      <c r="B40" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>32</v>
+      </c>
+      <c r="B41" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B42" s="15"/>
+      <c r="A42" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>230</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>32</v>
+        <v>124</v>
       </c>
       <c r="B44" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>137</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>139</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="B46" t="s">
-        <v>235</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>124</v>
+        <v>193</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>229</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>137</v>
+        <v>197</v>
       </c>
       <c r="B48" t="s">
-        <v>139</v>
+        <v>199</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="B49" t="s">
-        <v>140</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>193</v>
+        <v>225</v>
       </c>
       <c r="B50" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>197</v>
-      </c>
-      <c r="B51" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>207</v>
-      </c>
-      <c r="B52" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>230</v>
-      </c>
-      <c r="B53" t="s">
-        <v>231</v>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="B54" s="15"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>245</v>
+      </c>
+      <c r="B56" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="B57" s="15"/>
+      <c r="A57" t="s">
+        <v>246</v>
+      </c>
+      <c r="B57" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>248</v>
+      </c>
+      <c r="B58" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>250</v>
-      </c>
-      <c r="B59" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>251</v>
-      </c>
-      <c r="B60" t="s">
-        <v>256</v>
-      </c>
-    </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>253</v>
-      </c>
-      <c r="B61" t="s">
-        <v>254</v>
+      <c r="A61" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="15"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>6</v>
+      </c>
+      <c r="B62" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B64" s="15"/>
+      <c r="A64" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>6</v>
-      </c>
-      <c r="B65" t="s">
-        <v>228</v>
+        <v>59</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
         <v>72</v>
       </c>
     </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="B73" s="15"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A42:B42"/>
+  <mergeCells count="8">
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A61:B61"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A54:B54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added: policy checks on author/maintainer
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DF5C45-7E3C-4094-B8CA-4ED0D988DF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDD4AB9-1BE3-46A2-B4AE-9F6E8E8B7528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1755" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="29580" yWindow="2655" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="261">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -911,6 +911,18 @@
   </si>
   <si>
     <t>Recommended to specify author/maintainer to communicate on the dataset</t>
+  </si>
+  <si>
+    <t>Assist</t>
+  </si>
+  <si>
+    <t>Perform minimum changes and detect field types locally</t>
+  </si>
+  <si>
+    <t>CKAN DataStore merge</t>
+  </si>
+  <si>
+    <t>Merge existing DataStores on current CKAN (not tested)</t>
   </si>
 </sst>
 </file>
@@ -3340,6 +3352,14 @@
         <v>226</v>
       </c>
     </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>259</v>
+      </c>
+      <c r="B51" t="s">
+        <v>260</v>
+      </c>
+    </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
         <v>243</v>
@@ -3373,6 +3393,14 @@
       </c>
       <c r="B58" t="s">
         <v>249</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>257</v>
+      </c>
+      <c r="B59" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added: get_datastore_dump_url renamed: set_limits_per_request fixed: multiple bugs thanks to various tests
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDD4AB9-1BE3-46A2-B4AE-9F6E8E8B7528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6628C78B-34FB-478C-BE97-AB9B1CEA3CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="2655" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -859,9 +859,6 @@
     <t>Time between each request in seconds</t>
   </si>
   <si>
-    <t>Limit</t>
-  </si>
-  <si>
     <t>Maximum number of records to return/send per request</t>
   </si>
   <si>
@@ -923,6 +920,9 @@
   </si>
   <si>
     <t>Merge existing DataStores on current CKAN (not tested)</t>
+  </si>
+  <si>
+    <t>Limit per request</t>
   </si>
 </sst>
 </file>
@@ -1490,13 +1490,13 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="B10">
         <v>1000</v>
       </c>
       <c r="C10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2272,13 +2272,13 @@
     </row>
     <row r="2" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D2" s="14" t="str">
         <f>HYPERLINK(IF(RIGHT(CKAN_URL,1)="/", CKAN_URL &amp; "dataset/" &amp; package_name, CKAN_URL &amp; "/dataset/" &amp; package_name))</f>
@@ -2371,7 +2371,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2384,7 +2384,7 @@
         <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2482,7 +2482,7 @@
         <v>98</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>208</v>
@@ -3196,15 +3196,15 @@
         <v>219</v>
       </c>
       <c r="B18" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>251</v>
+      </c>
+      <c r="B19" t="s">
         <v>252</v>
-      </c>
-      <c r="B19" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3354,53 +3354,53 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>258</v>
+      </c>
+      <c r="B51" t="s">
         <v>259</v>
-      </c>
-      <c r="B51" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B54" s="15"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B56" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B57" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>247</v>
+      </c>
+      <c r="B58" t="s">
         <v>248</v>
-      </c>
-      <c r="B58" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>256</v>
+      </c>
+      <c r="B59" t="s">
         <v>257</v>
-      </c>
-      <c r="B59" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -3444,7 +3444,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="15" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B73" s="15"/>
     </row>

</xml_diff>

<commit_message>
doc: documentation in example Excel workbook
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6628C78B-34FB-478C-BE97-AB9B1CEA3CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FF2351-5ABA-4E89-9C07-0D1022789CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="12645" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="263">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -923,6 +923,12 @@
   </si>
   <si>
     <t>Limit per request</t>
+  </si>
+  <si>
+    <t>Maximum number of lines in each request.</t>
+  </si>
+  <si>
+    <t>Delay between requests, in seconds.</t>
   </si>
 </sst>
 </file>
@@ -1518,7 +1524,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24566A16-C143-4E07-9D41-A5CDAE0B0792}">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" style="5" bestFit="1" customWidth="1"/>
@@ -1645,7 +1651,7 @@
         <v>53</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>1</v>
+        <v>240</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>147</v>
@@ -1902,123 +1908,123 @@
         <v>224</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="20" t="s">
+      <c r="B40" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="C38" s="20"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="C40" s="20"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="375" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>187</v>
+        <v>46</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="375" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>47</v>
+        <v>187</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="90" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -2026,92 +2032,92 @@
         <v>54</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B50" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C52" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="12" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="21" t="s">
+      <c r="B53" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="C51" s="21"/>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="6" t="s">
+      <c r="C53" s="21"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B52" s="22" t="s">
+      <c r="B54" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="C52" s="22"/>
-    </row>
-    <row r="53" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
+      <c r="C54" s="22"/>
+    </row>
+    <row r="55" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B53" s="19" t="s">
+      <c r="B55" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="C53" s="19"/>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C55" s="9" t="s">
-        <v>132</v>
-      </c>
+      <c r="C55" s="19"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>111</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>162</v>
+        <v>79</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="90" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>111</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>191</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -2119,10 +2125,10 @@
         <v>111</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>211</v>
+        <v>162</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>214</v>
+        <v>163</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -2130,10 +2136,10 @@
         <v>111</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>212</v>
+        <v>3</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>215</v>
+        <v>191</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -2141,9 +2147,31 @@
         <v>111</v>
       </c>
       <c r="B60" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B62" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C62" s="9" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2152,13 +2180,13 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B55:C55"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed: load Excel workbook with non-existing resources directory added: user can programmatically configure arguments to pass to the upload/download functions: mapper_kwargs updated: example Excel workbook to list new file formats, doc
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FF2351-5ABA-4E89-9C07-0D1022789CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F14FBA2-BD66-46F6-8AE2-A52C7C15C5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="12645" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="28680" yWindow="1755" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="270">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -898,9 +898,6 @@
     <t>geometry(GEOMETRY,4326)</t>
   </si>
   <si>
-    <t>Field accepting GeoJSON (WKB hexadecimal preferred), in WGS84 coordinate system</t>
-  </si>
-  <si>
     <t>Binary JSON</t>
   </si>
   <si>
@@ -929,6 +926,30 @@
   </si>
   <si>
     <t>Delay between requests, in seconds.</t>
+  </si>
+  <si>
+    <t>PARQUET</t>
+  </si>
+  <si>
+    <t>GEOPARQUET</t>
+  </si>
+  <si>
+    <t>XLS</t>
+  </si>
+  <si>
+    <t>JSON (might need further customization of arguments)</t>
+  </si>
+  <si>
+    <t>SHP</t>
+  </si>
+  <si>
+    <t>Shape file</t>
+  </si>
+  <si>
+    <t>PNG</t>
+  </si>
+  <si>
+    <t>Field accepting GeoJSON (WKB hexadecimal preferred), in WGS84 coordinate system (4326). To convert from an existing EPSG, use argument --epsg-src in the Options column of the field</t>
   </si>
 </sst>
 </file>
@@ -1496,7 +1517,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B10">
         <v>1000</v>
@@ -1913,10 +1934,10 @@
         <v>109</v>
       </c>
       <c r="B38" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="C38" s="9" t="s">
         <v>260</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1927,7 +1948,7 @@
         <v>237</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -2399,7 +2420,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2412,7 +2433,7 @@
         <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2703,7 +2724,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{ABB3E20A-99D1-46AC-9089-895EB5CEC278}">
           <x14:formula1>
-            <xm:f>validation!$A$62:$A$72</xm:f>
+            <xm:f>validation!$A$62:$A$77</xm:f>
           </x14:formula1>
           <xm:sqref>C1:C1048576</xm:sqref>
         </x14:dataValidation>
@@ -3141,7 +3162,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397C6D0D-9607-4B06-96F5-66D1EA23B080}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B78"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -3224,7 +3245,7 @@
         <v>219</v>
       </c>
       <c r="B18" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3232,7 +3253,7 @@
         <v>251</v>
       </c>
       <c r="B19" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3382,10 +3403,10 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>257</v>
+      </c>
+      <c r="B51" t="s">
         <v>258</v>
-      </c>
-      <c r="B51" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -3425,10 +3446,10 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>255</v>
+      </c>
+      <c r="B59" t="s">
         <v>256</v>
-      </c>
-      <c r="B59" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -3447,38 +3468,69 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>13</v>
+        <v>59</v>
+      </c>
+      <c r="B63" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>266</v>
+      </c>
+      <c r="B64" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>59</v>
+        <v>262</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>71</v>
+        <v>263</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="15" t="s">
-        <v>254</v>
-      </c>
-      <c r="B73" s="15"/>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="B78" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A78:B78"/>
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A13:B13"/>

</xml_diff>